<commit_message>
lstm trained and save weight
</commit_message>
<xml_diff>
--- a/MRP_AI_Predictions.xlsx
+++ b/MRP_AI_Predictions.xlsx
@@ -516,7 +516,7 @@
         <v>6</v>
       </c>
       <c r="B2">
-        <v>153.4328460693359</v>
+        <v>152.2281341552734</v>
       </c>
       <c r="C2">
         <v>25</v>
@@ -528,7 +528,7 @@
         <v>60</v>
       </c>
       <c r="F2">
-        <v>76.43284606933594</v>
+        <v>75.22813415527344</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -536,7 +536,7 @@
         <v>7</v>
       </c>
       <c r="B3">
-        <v>158.7920532226562</v>
+        <v>157.7231140136719</v>
       </c>
       <c r="C3">
         <v>20</v>
@@ -548,7 +548,7 @@
         <v>80</v>
       </c>
       <c r="F3">
-        <v>80.79205322265625</v>
+        <v>79.72311401367188</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -556,7 +556,7 @@
         <v>8</v>
       </c>
       <c r="B4">
-        <v>302.7594299316406</v>
+        <v>315.9134216308594</v>
       </c>
       <c r="C4">
         <v>250</v>
@@ -568,7 +568,7 @@
         <v>500</v>
       </c>
       <c r="F4">
-        <v>-22.24057006835938</v>
+        <v>-9.086578369140625</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -576,7 +576,7 @@
         <v>9</v>
       </c>
       <c r="B5">
-        <v>152.9817657470703</v>
+        <v>151.5955505371094</v>
       </c>
       <c r="C5">
         <v>25</v>
@@ -588,7 +588,7 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>135.9817657470703</v>
+        <v>134.5955505371094</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -596,7 +596,7 @@
         <v>10</v>
       </c>
       <c r="B6">
-        <v>153.0236511230469</v>
+        <v>151.7098388671875</v>
       </c>
       <c r="C6">
         <v>25</v>
@@ -608,7 +608,7 @@
         <v>0</v>
       </c>
       <c r="F6">
-        <v>136.0236511230469</v>
+        <v>134.7098388671875</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -616,7 +616,7 @@
         <v>11</v>
       </c>
       <c r="B7">
-        <v>153.1784210205078</v>
+        <v>151.8041076660156</v>
       </c>
       <c r="C7">
         <v>25</v>
@@ -628,7 +628,7 @@
         <v>0</v>
       </c>
       <c r="F7">
-        <v>136.1784210205078</v>
+        <v>134.8041076660156</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -636,7 +636,7 @@
         <v>12</v>
       </c>
       <c r="B8">
-        <v>152.4496459960938</v>
+        <v>151.3575897216797</v>
       </c>
       <c r="C8">
         <v>25</v>
@@ -648,7 +648,7 @@
         <v>0</v>
       </c>
       <c r="F8">
-        <v>135.4496459960938</v>
+        <v>134.3575897216797</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -656,7 +656,7 @@
         <v>13</v>
       </c>
       <c r="B9">
-        <v>153.0320739746094</v>
+        <v>151.80029296875</v>
       </c>
       <c r="C9">
         <v>25</v>
@@ -668,7 +668,7 @@
         <v>0</v>
       </c>
       <c r="F9">
-        <v>136.0320739746094</v>
+        <v>134.80029296875</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -676,7 +676,7 @@
         <v>14</v>
       </c>
       <c r="B10">
-        <v>152.7441558837891</v>
+        <v>151.5839385986328</v>
       </c>
       <c r="C10">
         <v>25</v>
@@ -688,7 +688,7 @@
         <v>0</v>
       </c>
       <c r="F10">
-        <v>135.7441558837891</v>
+        <v>134.5839385986328</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -696,7 +696,7 @@
         <v>15</v>
       </c>
       <c r="B11">
-        <v>153.5006256103516</v>
+        <v>151.9650268554688</v>
       </c>
       <c r="C11">
         <v>25</v>
@@ -708,7 +708,7 @@
         <v>0</v>
       </c>
       <c r="F11">
-        <v>136.5006256103516</v>
+        <v>134.9650268554688</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -716,7 +716,7 @@
         <v>16</v>
       </c>
       <c r="B12">
-        <v>152.7609405517578</v>
+        <v>151.5505676269531</v>
       </c>
       <c r="C12">
         <v>25</v>
@@ -728,7 +728,7 @@
         <v>0</v>
       </c>
       <c r="F12">
-        <v>135.7609405517578</v>
+        <v>134.5505676269531</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -736,7 +736,7 @@
         <v>17</v>
       </c>
       <c r="B13">
-        <v>153.5470886230469</v>
+        <v>151.8899536132812</v>
       </c>
       <c r="C13">
         <v>25</v>
@@ -748,7 +748,7 @@
         <v>0</v>
       </c>
       <c r="F13">
-        <v>136.5470886230469</v>
+        <v>134.8899536132812</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -756,7 +756,7 @@
         <v>18</v>
       </c>
       <c r="B14">
-        <v>152.7333984375</v>
+        <v>151.6146850585938</v>
       </c>
       <c r="C14">
         <v>25</v>
@@ -768,7 +768,7 @@
         <v>0</v>
       </c>
       <c r="F14">
-        <v>135.7333984375</v>
+        <v>134.6146850585938</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -776,7 +776,7 @@
         <v>19</v>
       </c>
       <c r="B15">
-        <v>158.0364685058594</v>
+        <v>156.8740539550781</v>
       </c>
       <c r="C15">
         <v>20</v>
@@ -788,7 +788,7 @@
         <v>20</v>
       </c>
       <c r="F15">
-        <v>140.0364685058594</v>
+        <v>138.8740539550781</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -796,7 +796,7 @@
         <v>20</v>
       </c>
       <c r="B16">
-        <v>157.5316925048828</v>
+        <v>156.6345367431641</v>
       </c>
       <c r="C16">
         <v>20</v>
@@ -808,7 +808,7 @@
         <v>20</v>
       </c>
       <c r="F16">
-        <v>139.5316925048828</v>
+        <v>138.6345367431641</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -816,7 +816,7 @@
         <v>21</v>
       </c>
       <c r="B17">
-        <v>157.7234039306641</v>
+        <v>156.6550750732422</v>
       </c>
       <c r="C17">
         <v>20</v>
@@ -828,7 +828,7 @@
         <v>20</v>
       </c>
       <c r="F17">
-        <v>139.7234039306641</v>
+        <v>138.6550750732422</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -836,7 +836,7 @@
         <v>22</v>
       </c>
       <c r="B18">
-        <v>157.3439025878906</v>
+        <v>156.6184997558594</v>
       </c>
       <c r="C18">
         <v>20</v>
@@ -848,7 +848,7 @@
         <v>20</v>
       </c>
       <c r="F18">
-        <v>139.3439025878906</v>
+        <v>138.6184997558594</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -856,7 +856,7 @@
         <v>23</v>
       </c>
       <c r="B19">
-        <v>157.4517822265625</v>
+        <v>156.6291809082031</v>
       </c>
       <c r="C19">
         <v>20</v>
@@ -868,7 +868,7 @@
         <v>20</v>
       </c>
       <c r="F19">
-        <v>139.4517822265625</v>
+        <v>138.6291809082031</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -876,7 +876,7 @@
         <v>24</v>
       </c>
       <c r="B20">
-        <v>157.6978454589844</v>
+        <v>156.7843627929688</v>
       </c>
       <c r="C20">
         <v>20</v>
@@ -888,7 +888,7 @@
         <v>20</v>
       </c>
       <c r="F20">
-        <v>139.6978454589844</v>
+        <v>138.7843627929688</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -896,7 +896,7 @@
         <v>25</v>
       </c>
       <c r="B21">
-        <v>157.5846862792969</v>
+        <v>156.6518249511719</v>
       </c>
       <c r="C21">
         <v>20</v>
@@ -908,7 +908,7 @@
         <v>20</v>
       </c>
       <c r="F21">
-        <v>139.5846862792969</v>
+        <v>138.6518249511719</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -916,7 +916,7 @@
         <v>26</v>
       </c>
       <c r="B22">
-        <v>157.5492248535156</v>
+        <v>156.6193389892578</v>
       </c>
       <c r="C22">
         <v>20</v>
@@ -928,7 +928,7 @@
         <v>20</v>
       </c>
       <c r="F22">
-        <v>139.5492248535156</v>
+        <v>138.6193389892578</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -936,7 +936,7 @@
         <v>27</v>
       </c>
       <c r="B23">
-        <v>157.6785430908203</v>
+        <v>156.703125</v>
       </c>
       <c r="C23">
         <v>20</v>
@@ -948,7 +948,7 @@
         <v>20</v>
       </c>
       <c r="F23">
-        <v>139.6785430908203</v>
+        <v>138.703125</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -956,7 +956,7 @@
         <v>28</v>
       </c>
       <c r="B24">
-        <v>157.8500823974609</v>
+        <v>156.7980346679688</v>
       </c>
       <c r="C24">
         <v>20</v>
@@ -968,7 +968,7 @@
         <v>20</v>
       </c>
       <c r="F24">
-        <v>139.8500823974609</v>
+        <v>138.7980346679688</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -976,7 +976,7 @@
         <v>29</v>
       </c>
       <c r="B25">
-        <v>295.937744140625</v>
+        <v>309.4971618652344</v>
       </c>
       <c r="C25">
         <v>250</v>
@@ -988,7 +988,7 @@
         <v>300</v>
       </c>
       <c r="F25">
-        <v>170.937744140625</v>
+        <v>184.4971618652344</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -996,7 +996,7 @@
         <v>30</v>
       </c>
       <c r="B26">
-        <v>328.7368774414062</v>
+        <v>356.6873474121094</v>
       </c>
       <c r="C26">
         <v>250</v>
@@ -1008,7 +1008,7 @@
         <v>300</v>
       </c>
       <c r="F26">
-        <v>203.7368774414062</v>
+        <v>231.6873474121094</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -1016,7 +1016,7 @@
         <v>31</v>
       </c>
       <c r="B27">
-        <v>329.1467590332031</v>
+        <v>357.426513671875</v>
       </c>
       <c r="C27">
         <v>250</v>
@@ -1028,7 +1028,7 @@
         <v>300</v>
       </c>
       <c r="F27">
-        <v>204.1467590332031</v>
+        <v>232.426513671875</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -1036,7 +1036,7 @@
         <v>32</v>
       </c>
       <c r="B28">
-        <v>356.8616638183594</v>
+        <v>397.2751159667969</v>
       </c>
       <c r="C28">
         <v>250</v>
@@ -1048,7 +1048,7 @@
         <v>300</v>
       </c>
       <c r="F28">
-        <v>231.8616638183594</v>
+        <v>272.2751159667969</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -1056,7 +1056,7 @@
         <v>33</v>
       </c>
       <c r="B29">
-        <v>295.7943115234375</v>
+        <v>309.1565856933594</v>
       </c>
       <c r="C29">
         <v>250</v>
@@ -1068,7 +1068,7 @@
         <v>300</v>
       </c>
       <c r="F29">
-        <v>170.7943115234375</v>
+        <v>184.1565856933594</v>
       </c>
     </row>
     <row r="30" spans="1:6">
@@ -1076,7 +1076,7 @@
         <v>34</v>
       </c>
       <c r="B30">
-        <v>328.1439514160156</v>
+        <v>354.9096984863281</v>
       </c>
       <c r="C30">
         <v>250</v>
@@ -1088,7 +1088,7 @@
         <v>300</v>
       </c>
       <c r="F30">
-        <v>203.1439514160156</v>
+        <v>229.9096984863281</v>
       </c>
     </row>
     <row r="31" spans="1:6">
@@ -1096,7 +1096,7 @@
         <v>35</v>
       </c>
       <c r="B31">
-        <v>328.3083190917969</v>
+        <v>355.4646911621094</v>
       </c>
       <c r="C31">
         <v>250</v>
@@ -1108,7 +1108,7 @@
         <v>300</v>
       </c>
       <c r="F31">
-        <v>203.3083190917969</v>
+        <v>230.4646911621094</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -1116,7 +1116,7 @@
         <v>36</v>
       </c>
       <c r="B32">
-        <v>329.407470703125</v>
+        <v>356.3917846679688</v>
       </c>
       <c r="C32">
         <v>250</v>
@@ -1128,7 +1128,7 @@
         <v>300</v>
       </c>
       <c r="F32">
-        <v>204.407470703125</v>
+        <v>231.3917846679688</v>
       </c>
     </row>
     <row r="33" spans="1:6">
@@ -1136,7 +1136,7 @@
         <v>37</v>
       </c>
       <c r="B33">
-        <v>297.2477111816406</v>
+        <v>310.7924194335938</v>
       </c>
       <c r="C33">
         <v>250</v>
@@ -1148,7 +1148,7 @@
         <v>300</v>
       </c>
       <c r="F33">
-        <v>172.2477111816406</v>
+        <v>185.7924194335938</v>
       </c>
     </row>
     <row r="34" spans="1:6">
@@ -1156,7 +1156,7 @@
         <v>38</v>
       </c>
       <c r="B34">
-        <v>296.6250915527344</v>
+        <v>310.2366638183594</v>
       </c>
       <c r="C34">
         <v>250</v>
@@ -1168,7 +1168,7 @@
         <v>300</v>
       </c>
       <c r="F34">
-        <v>171.6250915527344</v>
+        <v>185.2366638183594</v>
       </c>
     </row>
   </sheetData>

</xml_diff>